<commit_message>
Added fields to templates and query.
</commit_message>
<xml_diff>
--- a/api/templates/genxpert_tb_workload_report/uk.xlsx
+++ b/api/templates/genxpert_tb_workload_report/uk.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25629"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-18.04\home\nsabaj\Repositories\aspect\api\templates\device_report\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\ubuntu\home\ahernandez\repos\aspect\api\templates\genxpert_tb_workload_report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AEE26AC-C6DA-4E32-BF7C-1AE56613DE14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{123666AA-145F-4000-8D69-C13B35621A98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-60" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="24" yWindow="24" windowWidth="23016" windowHeight="12936" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Devices" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="64">
   <si>
     <t>Пристрої GeneXpert</t>
   </si>
@@ -206,9 +206,6 @@
     <t>&lt;reasonForInterruption&gt;</t>
   </si>
   <si>
-    <t>&lt;totalXpertTests&gt;</t>
-  </si>
-  <si>
     <t># MTB траса</t>
   </si>
   <si>
@@ -216,6 +213,21 @@
   </si>
   <si>
     <t># MTB+ Стійкий до RIF</t>
+  </si>
+  <si>
+    <t>&lt;lastResultUploadedOn&gt;</t>
+  </si>
+  <si>
+    <t>&lt;lastResultConductedOn&gt;</t>
+  </si>
+  <si>
+    <t>&lt;totalXpertResults&gt;</t>
+  </si>
+  <si>
+    <t>Останній результат завантажено на</t>
+  </si>
+  <si>
+    <t>Останній результат проведено на</t>
   </si>
 </sst>
 </file>
@@ -225,7 +237,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -258,6 +270,14 @@
     </font>
     <font>
       <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <u/>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -321,8 +341,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -331,9 +350,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -356,6 +372,11 @@
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -738,7 +759,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AA14"/>
+  <dimension ref="A1:AC14"/>
   <sheetFormatPr defaultColWidth="11.296875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27.19921875" customWidth="1"/>
@@ -751,246 +772,264 @@
     <col min="14" max="14" width="13.59765625" customWidth="1"/>
     <col min="15" max="21" width="15.59765625" customWidth="1"/>
     <col min="22" max="23" width="20.59765625" customWidth="1"/>
-    <col min="24" max="25" width="20.59765625" style="2" customWidth="1"/>
+    <col min="24" max="25" width="20.59765625" style="1" customWidth="1"/>
     <col min="26" max="26" width="33.296875" customWidth="1"/>
-    <col min="27" max="27" width="20.59765625" customWidth="1"/>
+    <col min="27" max="27" width="32.8984375" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="31.09765625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="20.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" ht="21" x14ac:dyDescent="0.4">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:29" ht="21" x14ac:dyDescent="0.4">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-    </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+    </row>
+    <row r="2" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="18" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="1"/>
-    </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="D3" s="16"/>
+    </row>
+    <row r="4" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
+    <row r="5" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="18" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:27" ht="78" x14ac:dyDescent="0.3">
-      <c r="C6" s="5" t="s">
+    <row r="6" spans="1:29" ht="47.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="17" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="A7" s="7"/>
-    </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="A8" s="8"/>
-    </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.3">
+      <c r="E6" s="17"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="17"/>
+    </row>
+    <row r="7" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="A7" s="5"/>
+    </row>
+    <row r="8" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="A8" s="6"/>
+    </row>
+    <row r="9" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:27" s="12" customFormat="1" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A10" s="9" t="s">
+    <row r="10" spans="1:29" s="10" customFormat="1" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="D10" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="9" t="s">
+      <c r="E10" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="G10" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="H10" s="9" t="s">
+      <c r="H10" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="J10" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="K10" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="L10" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="I10" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="J10" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="K10" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="L10" s="10" t="s">
+      <c r="M10" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="M10" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="N10" s="9" t="s">
+      <c r="N10" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="O10" s="9" t="s">
+      <c r="O10" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="P10" s="9" t="s">
+      <c r="P10" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="Q10" s="9" t="s">
+      <c r="Q10" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="R10" s="9" t="s">
+      <c r="R10" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="S10" s="9" t="s">
+      <c r="S10" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="T10" s="9" t="s">
+      <c r="T10" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="U10" s="10" t="s">
+      <c r="U10" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="V10" s="10" t="s">
+      <c r="V10" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="W10" s="9" t="s">
+      <c r="W10" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="X10" s="11" t="s">
+      <c r="X10" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="Y10" s="11" t="s">
+      <c r="Y10" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="Z10" s="9" t="s">
+      <c r="Z10" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="AA10" s="9" t="s">
+      <c r="AA10" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="AB10" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="AC10" s="7" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="A11" s="13" t="s">
+    <row r="11" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="A11" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B11" s="13" t="s">
+      <c r="B11" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="D11" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="E11" s="13" t="s">
+      <c r="E11" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="F11" s="13" t="s">
+      <c r="F11" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="G11" s="13" t="s">
+      <c r="G11" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="H11" s="13" t="s">
+      <c r="H11" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="I11" s="14" t="s">
+      <c r="I11" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="J11" s="14" t="s">
+      <c r="J11" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="K11" s="14" t="s">
+      <c r="K11" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="L11" s="13" t="s">
+      <c r="L11" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="M11" s="13" t="s">
+      <c r="M11" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="N11" s="13" t="s">
+      <c r="N11" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="O11" s="14" t="s">
+      <c r="O11" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="P11" s="14" t="s">
+      <c r="P11" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="Q11" s="14" t="s">
+      <c r="Q11" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="R11" s="14" t="s">
+      <c r="R11" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="S11" s="14" t="s">
+      <c r="S11" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="T11" s="14" t="s">
+      <c r="T11" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="U11" s="13" t="s">
+      <c r="U11" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="V11" s="13" t="s">
+      <c r="V11" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="W11" s="13" t="s">
+      <c r="W11" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="X11" s="15" t="e">
-        <f>IF(AA11=0,0,I11/AA11)</f>
+      <c r="X11" s="13" t="e">
+        <f>IF(AC11=0,0,I11/AC11)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="Y11" s="16" t="e">
-        <f>IF(AA11=0,0,(I11+J11)/AA11)</f>
+      <c r="Y11" s="14" t="e">
+        <f>IF(AC11=0,0,(I11+J11)/AC11)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="Z11" s="16" t="e">
+      <c r="Z11" s="14" t="e">
         <f>IF(Y11&gt;0.05,"Високий рівень помилок/недійсних даних. Звертайтесь до лаб.","")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="AA11" s="13" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="B14" s="17"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
+      <c r="AA11" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="AB11" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="AC11" s="11" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="14" spans="1:29" x14ac:dyDescent="0.3">
+      <c r="B14" s="15"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="C3:D3"/>
+    <mergeCell ref="D6:G6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>